<commit_message>
Feat: -Massive update adding payroll -Update workload abc document
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/Documents/Blank_workload.xlsx
+++ b/SupervisorMobility.API/Documents/Blank_workload.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikoG\Documents\GrupoSinco\Cargas De Trabajo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikoG\Documents\GrupoSinco\SupervisorMobility\SupervisorMobility.API\SupervisorMobility.API\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D486DFE-11CF-4DE7-927B-003E9900CEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10FEA7AA-1CA3-4D13-8BE6-D822E8E99825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1275" yWindow="255" windowWidth="36120" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19920" yWindow="-14160" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Distribution" sheetId="9" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Carga de Trabajo por Modelo</t>
   </si>
@@ -102,6 +102,12 @@
   </si>
   <si>
     <t>ALL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DS Relevant / Imp ABC </t>
+  </si>
+  <si>
+    <t>Importante ABC</t>
   </si>
 </sst>
 </file>
@@ -213,7 +219,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="59">
+  <borders count="61">
     <border>
       <left/>
       <right/>
@@ -985,11 +991,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1117,6 +1147,138 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1165,136 +1327,25 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1363,10 +1414,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>447024</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>24894</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>447023</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>98163</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="7596693" cy="4303135"/>
     <xdr:pic>
@@ -1390,7 +1441,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19573224" y="2025144"/>
+          <a:off x="24274177" y="1446317"/>
           <a:ext cx="7596693" cy="4303135"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2178,6 +2229,876 @@
         <a:xfrm>
           <a:off x="406460" y="19771247"/>
           <a:ext cx="323850" cy="269875"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>6</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4343202" cy="1181100"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{64702129-4813-405D-B440-EA54EA3729B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="619125" y="0"/>
+          <a:ext cx="4343202" cy="1181100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>436563</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>130969</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Isosceles Triangle 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB5F22D1-2010-4246-A91E-FEC69D07EB47}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="436563" y="6124575"/>
+          <a:ext cx="313531" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>2</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>430212</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>124618</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Isosceles Triangle 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{005038D3-DC5E-4D93-8D50-883DD7944239}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="430212" y="6124575"/>
+          <a:ext cx="313531" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>2</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>429070</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>143320</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Isosceles Triangle 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9D1FAB5-28D8-41B1-AA02-C815F8AB1671}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="429070" y="6124575"/>
+          <a:ext cx="333375" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>429070</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>143320</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="Isosceles Triangle 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{601BD1C2-99D0-4BFC-BADA-7BE38B427CC0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="429070" y="6124575"/>
+          <a:ext cx="333375" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>429070</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>143320</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="Isosceles Triangle 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7EA36EEB-994E-40C5-B22E-537D19B0100F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="429070" y="6124575"/>
+          <a:ext cx="333375" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>429070</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>143320</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="Isosceles Triangle 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E580895-22B0-45DC-9D47-0EEB5915C8C6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="429070" y="6124575"/>
+          <a:ext cx="333375" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>442564</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>156814</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="Isosceles Triangle 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{820E875E-2073-42AC-B359-E6EFE9DB9F49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="442564" y="6124575"/>
+          <a:ext cx="333375" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>184955</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>510208</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Isosceles Triangle 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68B675B6-BD0E-4937-96DF-E39866ADEF87}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="184955" y="6124575"/>
+          <a:ext cx="325253" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>412927</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>127177</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="Isosceles Triangle 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90A0CA8D-0FD8-453A-9B4D-9540D8B3321B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="412927" y="6124575"/>
+          <a:ext cx="333375" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>5</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>208869</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>518431</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="Isosceles Triangle 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D4F500BD-93E3-4428-9D81-E012D08C7D6A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="208869" y="6124575"/>
+          <a:ext cx="309562" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="triangle">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFC000"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>4</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>406460</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>111185</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="Isosceles Triangle 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D71FED63-3B2A-4BC8-BF05-0D6EA77460E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="406460" y="6124575"/>
+          <a:ext cx="323850" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="triangle">
           <a:avLst/>
@@ -2498,229 +3419,238 @@
     <col min="3" max="3" width="21.28515625" customWidth="1"/>
     <col min="4" max="4" width="46.7109375" customWidth="1"/>
     <col min="5" max="5" width="26.28515625" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" customWidth="1"/>
+    <col min="6" max="6" width="39.85546875" customWidth="1"/>
     <col min="7" max="24" width="8" customWidth="1"/>
     <col min="25" max="25" width="13.7109375" customWidth="1"/>
     <col min="26" max="26" width="15.7109375" customWidth="1"/>
-    <col min="27" max="28" width="6.7109375" customWidth="1"/>
+    <col min="27" max="27" width="26.7109375" customWidth="1"/>
+    <col min="28" max="28" width="6.7109375" customWidth="1"/>
     <col min="29" max="29" width="93.7109375" customWidth="1"/>
     <col min="30" max="30" width="9.42578125" customWidth="1"/>
     <col min="31" max="34" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:30" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="102"/>
-      <c r="D1" s="102"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="102"/>
-      <c r="G1" s="102"/>
-      <c r="H1" s="102"/>
-      <c r="I1" s="102"/>
-      <c r="J1" s="102"/>
-      <c r="K1" s="102"/>
-      <c r="L1" s="102"/>
-      <c r="M1" s="102"/>
-      <c r="N1" s="102"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="103" t="s">
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="Q1" s="105" t="s">
+      <c r="R1" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="105"/>
-      <c r="S1" s="105" t="s">
+      <c r="S1" s="50"/>
+      <c r="T1" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="105"/>
-      <c r="U1" s="105"/>
-      <c r="V1" s="105"/>
-      <c r="W1" s="105" t="s">
+      <c r="U1" s="50"/>
+      <c r="V1" s="50"/>
+      <c r="W1" s="50"/>
+      <c r="X1" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="X1" s="105"/>
-      <c r="Y1" s="105"/>
-      <c r="Z1" s="100" t="s">
+      <c r="Y1" s="50"/>
+      <c r="Z1" s="50"/>
+      <c r="AA1" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="AC1" s="96" t="s">
+      <c r="AC1" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="AD1" s="96"/>
+      <c r="AD1" s="54"/>
     </row>
     <row r="2" spans="2:30" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="102"/>
-      <c r="C2" s="102"/>
-      <c r="D2" s="102"/>
-      <c r="E2" s="102"/>
-      <c r="F2" s="102"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="102"/>
-      <c r="I2" s="102"/>
-      <c r="J2" s="102"/>
-      <c r="K2" s="102"/>
-      <c r="L2" s="102"/>
-      <c r="M2" s="102"/>
-      <c r="N2" s="102"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="104"/>
-      <c r="Q2" s="106"/>
-      <c r="R2" s="106"/>
-      <c r="S2" s="106"/>
-      <c r="T2" s="106"/>
-      <c r="U2" s="106"/>
-      <c r="V2" s="106"/>
-      <c r="W2" s="106"/>
-      <c r="X2" s="106"/>
-      <c r="Y2" s="106"/>
-      <c r="Z2" s="101"/>
-      <c r="AC2" s="96"/>
-      <c r="AD2" s="96"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="49"/>
+      <c r="R2" s="51"/>
+      <c r="S2" s="51"/>
+      <c r="T2" s="51"/>
+      <c r="U2" s="51"/>
+      <c r="V2" s="51"/>
+      <c r="W2" s="51"/>
+      <c r="X2" s="51"/>
+      <c r="Y2" s="51"/>
+      <c r="Z2" s="51"/>
+      <c r="AA2" s="59"/>
+      <c r="AC2" s="54"/>
+      <c r="AD2" s="54"/>
     </row>
     <row r="3" spans="2:30" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="41">
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="47"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="41">
         <v>1</v>
       </c>
-      <c r="Q3" s="97"/>
-      <c r="R3" s="97"/>
-      <c r="S3" s="97"/>
-      <c r="T3" s="97"/>
-      <c r="U3" s="97"/>
-      <c r="V3" s="97"/>
-      <c r="W3" s="98"/>
-      <c r="X3" s="99"/>
-      <c r="Y3" s="99"/>
-      <c r="Z3" s="42"/>
+      <c r="R3" s="55"/>
+      <c r="S3" s="55"/>
+      <c r="T3" s="55"/>
+      <c r="U3" s="55"/>
+      <c r="V3" s="55"/>
+      <c r="W3" s="55"/>
+      <c r="X3" s="56"/>
+      <c r="Y3" s="57"/>
+      <c r="Z3" s="57"/>
+      <c r="AA3" s="42"/>
     </row>
     <row r="4" spans="2:30" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="O4" s="3"/>
-      <c r="P4" s="29">
+      <c r="P4" s="3"/>
+      <c r="Q4" s="29">
         <v>2</v>
       </c>
-      <c r="Q4" s="78"/>
-      <c r="R4" s="78"/>
-      <c r="S4" s="78"/>
-      <c r="T4" s="78"/>
-      <c r="U4" s="78"/>
-      <c r="V4" s="78"/>
-      <c r="W4" s="80"/>
-      <c r="X4" s="78"/>
-      <c r="Y4" s="78"/>
-      <c r="Z4" s="4"/>
+      <c r="R4" s="53"/>
+      <c r="S4" s="53"/>
+      <c r="T4" s="53"/>
+      <c r="U4" s="53"/>
+      <c r="V4" s="53"/>
+      <c r="W4" s="53"/>
+      <c r="X4" s="52"/>
+      <c r="Y4" s="53"/>
+      <c r="Z4" s="53"/>
+      <c r="AA4" s="4"/>
     </row>
     <row r="5" spans="2:30" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="93" t="s">
+      <c r="B5" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="94"/>
+      <c r="C5" s="61"/>
       <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="107" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="93" t="s">
+      <c r="G5" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="95"/>
-      <c r="H5" s="95"/>
-      <c r="I5" s="94"/>
-      <c r="J5" s="93" t="s">
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="61"/>
+      <c r="K5" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="95"/>
-      <c r="L5" s="95"/>
-      <c r="M5" s="95"/>
-      <c r="N5" s="94"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="2">
+      <c r="L5" s="62"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
+      <c r="O5" s="61"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="2">
         <v>3</v>
       </c>
-      <c r="Q5" s="78"/>
-      <c r="R5" s="78"/>
-      <c r="S5" s="79"/>
-      <c r="T5" s="79"/>
-      <c r="U5" s="79"/>
-      <c r="V5" s="79"/>
-      <c r="W5" s="80"/>
-      <c r="X5" s="78"/>
-      <c r="Y5" s="78"/>
-      <c r="Z5" s="4"/>
+      <c r="R5" s="53"/>
+      <c r="S5" s="53"/>
+      <c r="T5" s="63"/>
+      <c r="U5" s="63"/>
+      <c r="V5" s="63"/>
+      <c r="W5" s="63"/>
+      <c r="X5" s="52"/>
+      <c r="Y5" s="53"/>
+      <c r="Z5" s="53"/>
+      <c r="AA5" s="4"/>
     </row>
     <row r="6" spans="2:30" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="81"/>
-      <c r="C6" s="82"/>
-      <c r="D6" s="85"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="86"/>
-      <c r="G6" s="88"/>
-      <c r="H6" s="88"/>
-      <c r="I6" s="89"/>
-      <c r="J6" s="92"/>
-      <c r="K6" s="88"/>
-      <c r="L6" s="88"/>
-      <c r="M6" s="88"/>
-      <c r="N6" s="89"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="29">
+      <c r="B6" s="64"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="108"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="71"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="72"/>
+      <c r="K6" s="75"/>
+      <c r="L6" s="71"/>
+      <c r="M6" s="71"/>
+      <c r="N6" s="71"/>
+      <c r="O6" s="72"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="29">
         <v>4</v>
       </c>
-      <c r="Q6" s="78"/>
-      <c r="R6" s="78"/>
-      <c r="S6" s="78"/>
-      <c r="T6" s="78"/>
-      <c r="U6" s="78"/>
-      <c r="V6" s="78"/>
-      <c r="W6" s="80"/>
-      <c r="X6" s="78"/>
-      <c r="Y6" s="78"/>
-      <c r="Z6" s="7"/>
+      <c r="R6" s="53"/>
+      <c r="S6" s="53"/>
+      <c r="T6" s="53"/>
+      <c r="U6" s="53"/>
+      <c r="V6" s="53"/>
+      <c r="W6" s="53"/>
+      <c r="X6" s="52"/>
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
+      <c r="AA6" s="7"/>
     </row>
     <row r="7" spans="2:30" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="83"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="87"/>
-      <c r="F7" s="87"/>
-      <c r="G7" s="90"/>
-      <c r="H7" s="90"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="87"/>
-      <c r="K7" s="90"/>
-      <c r="L7" s="90"/>
-      <c r="M7" s="90"/>
-      <c r="N7" s="91"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="2">
+      <c r="B7" s="66"/>
+      <c r="C7" s="67"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="109"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="70"/>
+      <c r="H7" s="73"/>
+      <c r="I7" s="73"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="70"/>
+      <c r="L7" s="73"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="74"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="2">
         <v>5</v>
       </c>
-      <c r="Q7" s="78"/>
-      <c r="R7" s="78"/>
-      <c r="S7" s="79"/>
-      <c r="T7" s="79"/>
-      <c r="U7" s="79"/>
-      <c r="V7" s="79"/>
-      <c r="W7" s="80"/>
-      <c r="X7" s="78"/>
-      <c r="Y7" s="78"/>
-      <c r="Z7" s="4"/>
+      <c r="R7" s="53"/>
+      <c r="S7" s="53"/>
+      <c r="T7" s="63"/>
+      <c r="U7" s="63"/>
+      <c r="V7" s="63"/>
+      <c r="W7" s="63"/>
+      <c r="X7" s="52"/>
+      <c r="Y7" s="53"/>
+      <c r="Z7" s="53"/>
+      <c r="AA7" s="4"/>
     </row>
     <row r="8" spans="2:30" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="43"/>
@@ -2736,138 +3666,144 @@
       <c r="L8" s="43"/>
       <c r="M8" s="43"/>
       <c r="N8" s="43"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="29">
+      <c r="O8" s="43"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="29">
         <v>6</v>
       </c>
-      <c r="Q8" s="78"/>
-      <c r="R8" s="78"/>
-      <c r="S8" s="79"/>
-      <c r="T8" s="79"/>
-      <c r="U8" s="79"/>
-      <c r="V8" s="79"/>
-      <c r="W8" s="80"/>
-      <c r="X8" s="78"/>
-      <c r="Y8" s="78"/>
-      <c r="Z8" s="7"/>
+      <c r="R8" s="53"/>
+      <c r="S8" s="53"/>
+      <c r="T8" s="63"/>
+      <c r="U8" s="63"/>
+      <c r="V8" s="63"/>
+      <c r="W8" s="63"/>
+      <c r="X8" s="52"/>
+      <c r="Y8" s="53"/>
+      <c r="Z8" s="53"/>
+      <c r="AA8" s="7"/>
     </row>
     <row r="9" spans="2:30" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="P9" s="44">
+      <c r="Q9" s="44">
         <v>7</v>
       </c>
-      <c r="Q9" s="63"/>
-      <c r="R9" s="63"/>
-      <c r="S9" s="64"/>
-      <c r="T9" s="64"/>
-      <c r="U9" s="64"/>
-      <c r="V9" s="64"/>
-      <c r="W9" s="65"/>
-      <c r="X9" s="63"/>
-      <c r="Y9" s="63"/>
-      <c r="Z9" s="31"/>
+      <c r="R9" s="76"/>
+      <c r="S9" s="76"/>
+      <c r="T9" s="77"/>
+      <c r="U9" s="77"/>
+      <c r="V9" s="77"/>
+      <c r="W9" s="77"/>
+      <c r="X9" s="78"/>
+      <c r="Y9" s="76"/>
+      <c r="Z9" s="76"/>
+      <c r="AA9" s="31"/>
     </row>
     <row r="10" spans="2:30" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="66"/>
-      <c r="C10" s="69" t="s">
+      <c r="B10" s="79"/>
+      <c r="C10" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="69" t="s">
+      <c r="D10" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="72" t="s">
+      <c r="E10" s="110" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="85" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="75" t="s">
+      <c r="G10" s="88" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="76"/>
-      <c r="J10" s="76"/>
-      <c r="K10" s="76"/>
-      <c r="L10" s="76"/>
-      <c r="M10" s="76"/>
-      <c r="N10" s="76"/>
-      <c r="O10" s="76"/>
-      <c r="P10" s="76"/>
-      <c r="Q10" s="76"/>
-      <c r="R10" s="76"/>
-      <c r="S10" s="76"/>
-      <c r="T10" s="76"/>
-      <c r="U10" s="76"/>
-      <c r="V10" s="76"/>
-      <c r="W10" s="76"/>
-      <c r="X10" s="76"/>
-      <c r="Y10" s="77"/>
-      <c r="Z10" s="56" t="s">
+      <c r="H10" s="89"/>
+      <c r="I10" s="89"/>
+      <c r="J10" s="89"/>
+      <c r="K10" s="89"/>
+      <c r="L10" s="89"/>
+      <c r="M10" s="89"/>
+      <c r="N10" s="89"/>
+      <c r="O10" s="89"/>
+      <c r="P10" s="89"/>
+      <c r="Q10" s="89"/>
+      <c r="R10" s="89"/>
+      <c r="S10" s="89"/>
+      <c r="T10" s="89"/>
+      <c r="U10" s="89"/>
+      <c r="V10" s="89"/>
+      <c r="W10" s="89"/>
+      <c r="X10" s="89"/>
+      <c r="Y10" s="89"/>
+      <c r="Z10" s="90"/>
+      <c r="AA10" s="100" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" spans="2:30" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="67"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="70"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="59" t="s">
+      <c r="B11" s="80"/>
+      <c r="C11" s="83"/>
+      <c r="D11" s="83"/>
+      <c r="E11" s="111"/>
+      <c r="F11" s="86"/>
+      <c r="G11" s="103" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="61"/>
-      <c r="K11" s="62" t="s">
+      <c r="H11" s="104"/>
+      <c r="I11" s="104"/>
+      <c r="J11" s="104"/>
+      <c r="K11" s="105"/>
+      <c r="L11" s="106" t="s">
         <v>15</v>
       </c>
-      <c r="L11" s="60"/>
-      <c r="M11" s="60"/>
-      <c r="N11" s="60"/>
-      <c r="O11" s="61"/>
-      <c r="P11" s="62" t="s">
+      <c r="M11" s="104"/>
+      <c r="N11" s="104"/>
+      <c r="O11" s="104"/>
+      <c r="P11" s="105"/>
+      <c r="Q11" s="106" t="s">
         <v>16</v>
       </c>
-      <c r="Q11" s="60"/>
-      <c r="R11" s="60"/>
-      <c r="S11" s="60"/>
-      <c r="T11" s="61"/>
-      <c r="U11" s="62"/>
-      <c r="V11" s="60"/>
-      <c r="W11" s="60"/>
-      <c r="X11" s="60"/>
-      <c r="Y11" s="61"/>
-      <c r="Z11" s="57"/>
+      <c r="R11" s="104"/>
+      <c r="S11" s="104"/>
+      <c r="T11" s="104"/>
+      <c r="U11" s="105"/>
+      <c r="V11" s="106"/>
+      <c r="W11" s="104"/>
+      <c r="X11" s="104"/>
+      <c r="Y11" s="104"/>
+      <c r="Z11" s="105"/>
+      <c r="AA11" s="101"/>
     </row>
     <row r="12" spans="2:30" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="68"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="74"/>
-      <c r="F12" s="8" t="s">
+      <c r="B12" s="81"/>
+      <c r="C12" s="84"/>
+      <c r="D12" s="84"/>
+      <c r="E12" s="112"/>
+      <c r="F12" s="87"/>
+      <c r="G12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="28"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="40"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="8" t="s">
+      <c r="H12" s="28"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="30"/>
+      <c r="L12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="L12" s="28"/>
-      <c r="M12" s="9"/>
+      <c r="M12" s="28"/>
       <c r="N12" s="9"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="8" t="s">
+      <c r="O12" s="9"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="Q12" s="28"/>
       <c r="R12" s="28"/>
-      <c r="S12" s="11"/>
-      <c r="T12" s="12"/>
-      <c r="U12" s="13"/>
-      <c r="V12" s="11"/>
+      <c r="S12" s="28"/>
+      <c r="T12" s="11"/>
+      <c r="U12" s="12"/>
+      <c r="V12" s="13"/>
       <c r="W12" s="11"/>
       <c r="X12" s="11"/>
-      <c r="Y12" s="12"/>
-      <c r="Z12" s="58"/>
+      <c r="Y12" s="11"/>
+      <c r="Z12" s="12"/>
+      <c r="AA12" s="102"/>
     </row>
     <row r="13" spans="2:30" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="32">
@@ -2875,29 +3811,28 @@
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="46"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="34"/>
-      <c r="H13" s="34"/>
+      <c r="E13" s="113"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="34"/>
       <c r="I13" s="34"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="34"/>
-      <c r="M13" s="36"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="35"/>
+      <c r="L13" s="33"/>
+      <c r="M13" s="34"/>
       <c r="N13" s="36"/>
-      <c r="O13" s="37"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="34"/>
-      <c r="R13" s="36"/>
+      <c r="O13" s="36"/>
+      <c r="P13" s="37"/>
+      <c r="Q13" s="33"/>
+      <c r="R13" s="34"/>
       <c r="S13" s="36"/>
-      <c r="T13" s="37"/>
-      <c r="U13" s="38"/>
-      <c r="V13" s="36"/>
+      <c r="T13" s="36"/>
+      <c r="U13" s="37"/>
+      <c r="V13" s="38"/>
       <c r="W13" s="36"/>
       <c r="X13" s="36"/>
-      <c r="Y13" s="37"/>
-      <c r="Z13" s="47">
-        <v>4</v>
-      </c>
+      <c r="Y13" s="36"/>
+      <c r="Z13" s="37"/>
+      <c r="AA13" s="91"/>
     </row>
     <row r="14" spans="2:30" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="32">
@@ -2905,27 +3840,28 @@
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="46"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="34"/>
+      <c r="E14" s="113"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="33"/>
       <c r="H14" s="34"/>
       <c r="I14" s="34"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="34"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="34"/>
-      <c r="O14" s="37"/>
-      <c r="P14" s="33"/>
-      <c r="Q14" s="34"/>
-      <c r="R14" s="36"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="34"/>
+      <c r="N14" s="36"/>
+      <c r="O14" s="34"/>
+      <c r="P14" s="37"/>
+      <c r="Q14" s="33"/>
+      <c r="R14" s="34"/>
       <c r="S14" s="36"/>
-      <c r="T14" s="37"/>
-      <c r="U14" s="38"/>
-      <c r="V14" s="36"/>
+      <c r="T14" s="36"/>
+      <c r="U14" s="37"/>
+      <c r="V14" s="38"/>
       <c r="W14" s="36"/>
       <c r="X14" s="36"/>
-      <c r="Y14" s="37"/>
-      <c r="Z14" s="48"/>
+      <c r="Y14" s="36"/>
+      <c r="Z14" s="37"/>
+      <c r="AA14" s="92"/>
     </row>
     <row r="15" spans="2:30" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="32">
@@ -2933,129 +3869,128 @@
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="46"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="34"/>
+      <c r="E15" s="113"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="36"/>
       <c r="I15" s="34"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="33"/>
-      <c r="L15" s="36"/>
+      <c r="J15" s="34"/>
+      <c r="K15" s="35"/>
+      <c r="L15" s="33"/>
       <c r="M15" s="36"/>
       <c r="N15" s="36"/>
-      <c r="O15" s="37"/>
-      <c r="P15" s="34"/>
-      <c r="R15" s="36"/>
+      <c r="O15" s="36"/>
+      <c r="P15" s="37"/>
+      <c r="Q15" s="34"/>
       <c r="S15" s="36"/>
-      <c r="T15" s="37"/>
-      <c r="U15" s="38"/>
-      <c r="V15" s="36"/>
+      <c r="T15" s="36"/>
+      <c r="U15" s="37"/>
+      <c r="V15" s="38"/>
       <c r="W15" s="36"/>
       <c r="X15" s="36"/>
-      <c r="Y15" s="37"/>
-      <c r="Z15" s="49"/>
+      <c r="Y15" s="36"/>
+      <c r="Z15" s="37"/>
+      <c r="AA15" s="93"/>
     </row>
     <row r="16" spans="2:30" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="50" t="s">
+      <c r="B16" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="51"/>
-      <c r="D16" s="51"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="16"/>
+      <c r="C16" s="95"/>
+      <c r="D16" s="95"/>
+      <c r="E16" s="95"/>
+      <c r="F16" s="96"/>
+      <c r="G16" s="15"/>
       <c r="H16" s="16"/>
       <c r="I16" s="16"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="45"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="18"/>
+      <c r="M16" s="19"/>
       <c r="N16" s="45"/>
       <c r="O16" s="45"/>
-      <c r="P16" s="18"/>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="20"/>
+      <c r="P16" s="45"/>
+      <c r="Q16" s="18"/>
+      <c r="R16" s="19"/>
       <c r="S16" s="20"/>
-      <c r="T16" s="21"/>
-      <c r="U16" s="22"/>
-      <c r="V16" s="23"/>
+      <c r="T16" s="20"/>
+      <c r="U16" s="21"/>
+      <c r="V16" s="22"/>
       <c r="W16" s="23"/>
       <c r="X16" s="23"/>
-      <c r="Y16" s="24"/>
-      <c r="Z16" s="39"/>
+      <c r="Y16" s="23"/>
+      <c r="Z16" s="24"/>
+      <c r="AA16" s="39"/>
     </row>
-    <row r="17" spans="2:26" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="53" t="s">
+    <row r="17" spans="2:27" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="25">
-        <f>SUM(F13:F16)</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="26">
+      <c r="C17" s="98"/>
+      <c r="D17" s="98"/>
+      <c r="E17" s="98"/>
+      <c r="F17" s="99"/>
+      <c r="G17" s="25">
         <f>SUM(G13:G16)</f>
         <v>0</v>
       </c>
       <c r="H17" s="26">
-        <f>SUM(H15:H16)</f>
+        <f>SUM(H13:H16)</f>
         <v>0</v>
       </c>
       <c r="I17" s="26">
         <f>SUM(I15:I16)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="27">
+      <c r="J17" s="26">
         <f>SUM(J15:J16)</f>
         <v>0</v>
       </c>
-      <c r="K17" s="25">
-        <f>SUM(K13:K16)</f>
+      <c r="K17" s="27">
+        <f>SUM(K15:K16)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="26">
+      <c r="L17" s="25">
         <f>SUM(L13:L16)</f>
         <v>0</v>
       </c>
       <c r="M17" s="26">
-        <f>SUM(M15:M16)</f>
+        <f>SUM(M13:M16)</f>
         <v>0</v>
       </c>
       <c r="N17" s="26">
         <f>SUM(N15:N16)</f>
         <v>0</v>
       </c>
-      <c r="O17" s="27">
+      <c r="O17" s="26">
         <f>SUM(O15:O16)</f>
         <v>0</v>
       </c>
-      <c r="P17" s="25">
-        <f>SUM(P13:P16)</f>
+      <c r="P17" s="27">
+        <f>SUM(P15:P16)</f>
         <v>0</v>
       </c>
-      <c r="Q17" s="26">
+      <c r="Q17" s="25">
         <f>SUM(Q13:Q16)</f>
         <v>0</v>
       </c>
       <c r="R17" s="26">
-        <f t="shared" ref="R17:Y17" si="0">SUM(R15:R16)</f>
+        <f>SUM(R13:R16)</f>
         <v>0</v>
       </c>
       <c r="S17" s="26">
+        <f t="shared" ref="S17:Z17" si="0">SUM(S15:S16)</f>
+        <v>0</v>
+      </c>
+      <c r="T17" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="T17" s="27">
+      <c r="U17" s="27">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="U17" s="25">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="V17" s="26">
+      <c r="V17" s="25">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3067,63 +4002,69 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Y17" s="27">
+      <c r="Y17" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Z17" s="39"/>
+      <c r="Z17" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AA17" s="39"/>
     </row>
   </sheetData>
-  <mergeCells count="49">
-    <mergeCell ref="B1:N3"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="Q1:R2"/>
-    <mergeCell ref="S1:V2"/>
-    <mergeCell ref="W1:Y2"/>
-    <mergeCell ref="W5:Y5"/>
-    <mergeCell ref="AC1:AD2"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="S3:V3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="S4:V4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z1:Z2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="J5:N5"/>
-    <mergeCell ref="Q5:R5"/>
-    <mergeCell ref="S5:V5"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="S8:V8"/>
-    <mergeCell ref="W8:Y8"/>
-    <mergeCell ref="B6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:I7"/>
-    <mergeCell ref="J6:N7"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="S6:V6"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="S7:V7"/>
-    <mergeCell ref="W7:Y7"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="S9:V9"/>
-    <mergeCell ref="W9:Y9"/>
+  <mergeCells count="51">
+    <mergeCell ref="AA13:AA15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="AA10:AA12"/>
+    <mergeCell ref="G11:K11"/>
+    <mergeCell ref="L11:P11"/>
+    <mergeCell ref="Q11:U11"/>
+    <mergeCell ref="V11:Z11"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="T8:W8"/>
+    <mergeCell ref="X8:Z8"/>
+    <mergeCell ref="R9:S9"/>
+    <mergeCell ref="T9:W9"/>
+    <mergeCell ref="X9:Z9"/>
+    <mergeCell ref="K6:O7"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="T6:W6"/>
+    <mergeCell ref="X6:Z6"/>
+    <mergeCell ref="R7:S7"/>
+    <mergeCell ref="T7:W7"/>
+    <mergeCell ref="X7:Z7"/>
+    <mergeCell ref="R4:S4"/>
+    <mergeCell ref="T4:W4"/>
+    <mergeCell ref="X4:Z4"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="K5:O5"/>
+    <mergeCell ref="R5:S5"/>
+    <mergeCell ref="T5:W5"/>
+    <mergeCell ref="X5:Z5"/>
+    <mergeCell ref="F10:F12"/>
+    <mergeCell ref="G10:Z10"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="C10:C12"/>
     <mergeCell ref="D10:D12"/>
     <mergeCell ref="E10:E12"/>
-    <mergeCell ref="F10:Y10"/>
-    <mergeCell ref="Z13:Z15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="Z10:Z12"/>
-    <mergeCell ref="F11:J11"/>
-    <mergeCell ref="K11:O11"/>
-    <mergeCell ref="P11:T11"/>
-    <mergeCell ref="U11:Y11"/>
+    <mergeCell ref="B6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:J7"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="AC1:AD2"/>
+    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="R1:S2"/>
+    <mergeCell ref="T1:W2"/>
+    <mergeCell ref="X1:Z2"/>
+    <mergeCell ref="AA1:AA2"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="T3:W3"/>
+    <mergeCell ref="B1:O3"/>
+    <mergeCell ref="X3:Z3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>